<commit_message>
Aplica correcciones del segundo corte al STRIDE (puntos 3, 4 y 5)
Sincroniza entrega/ con la versión corregida del repo de proyecto: OPAC existente,
Biteca como proveedor de Koha, estudiantes con cuentas compartidas, DFD con P1 y P2
en zonas externas y el formulario de Microsoft Forms, T3 y T6 recalculadas y nuevas
amenazas T7 a T9. Agrega el SVG del DFD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wXTRos7KirxghfoUX112D
</commit_message>
<xml_diff>
--- a/entrega/tabla-stride-cliente.xlsx
+++ b/entrega/tabla-stride-cliente.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La credencial es conocida por cualquier persona que haya trabajado en la biblioteca (sin proceso de revocación al cambiar de personal), o se filtra por phishing dirigido a la única bibliotecaria.</t>
+          <t>La credencial es conocida por cualquier persona que haya trabajado en la biblioteca (sin proceso de revocación al cambiar de personal) o se filtra por phishing dirigido a quien la usa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -591,57 +591,57 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Doble registro manual de datos personales (Koha y Llave del Saber)</t>
+          <t>Registro de acciones en Koha y Llave del Saber</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Tampering</t>
+          <t>Repudiation</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Al ingresarse manualmente el mismo dato dos veces sin validación cruzada automática, un error de digitación o una alteración intencional en una de las dos plataformas no es detectada por la otra.</t>
+          <t>Con cuentas compartidas (dos cuentas de Koha con permisos de edición que usan la bibliotecaria y los estudiantes de servicio social, y una credencial única por biblioteca en Llave del Saber), ninguna acción registrada puede atribuirse a una persona específica.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Alguien con acceso a una de las dos plataformas modifica un dato personal (ej. dirección o fecha de nacimiento) sin que exista mecanismo de reconciliación frente a la otra plataforma.</t>
+          <t>Un estudiante o la bibliotecaria modifica o elimina un registro de usuario o de catálogo con la cuenta compartida; el cambio no puede rastrearse a quien lo hizo ni demostrarse que no lo hizo. Esto ocurre hoy, no solo si se contrata un auxiliar.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Medio — inconsistencia de datos personales entre sistemas; dificulta auditoría y reportes al Ministerio</t>
+          <t>Alto: imposibilidad de auditar acciones individuales sobre datos personales (incluidos datos de menores) y de rendir cuentas ante la Alcaldía y la RNBP</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Alta: ya ocurre (estudiantes con cuentas compartidas, Taller 6 ítem 9)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Ninguno automatizado — la reconciliación depende completamente de una sola persona (cuello de botella ya diagnosticado en el Taller 4 de infraestructura).</t>
+          <t>Ninguno: Koha tiene cuentas compartidas contra lo que establece la política de la Alcaldía (num. 10) y Llave del Saber, por diseño, ofrece un único usuario por biblioteca (confirmado en el manual oficial).</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Definir un identificador único compartido (número de documento) y un proceso periódico de cruce de reportes entre ambas plataformas para detectar discrepancias.</t>
+          <t>Crear cuentas individuales en Koha, con perfil restringido para los estudiantes y baja al terminar el servicio social (Taller 6, ítem 9). En Llave del Saber, mientras no existan usuarios individuales, llevar una bitácora externa de quién trabaja cada sesión.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Bibliotecaria</t>
+          <t>Bibliotecaria / Alcaldía de Cogua / RNBP</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -653,57 +653,57 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Registro de acciones en Koha y Llave del Saber</t>
+          <t>Base de Datos Koha (Biteca) y Base de Datos Llave del Saber (RNBP)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Repudiation</t>
+          <t>Information Disclosure</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Al existir una única credencial compartida por biblioteca (no por persona), ninguna acción registrada puede atribuirse de forma inequívoca a una persona específica si llega a haber más de un empleado.</t>
+          <t>Ambas bases almacenan datos personales sensibles, incluyendo de menores de edad (categorías 'Niños 6-12' y 'Primera Infancia 0-5'), sin que el equipo tenga visibilidad de los controles de acceso y cifrado del proveedor externo.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Si se contrata el auxiliar que la bibliotecaria ya solicitó (ver ficha de caracterización), un cambio erróneo o malicioso en un registro no podría rastrearse a quién lo hizo, porque ambos entrarían con la misma cuenta institucional.</t>
+          <t>Una filtración en la infraestructura del proveedor externo (Biteca para Koha, o el Ministerio/RNBP para Llave del Saber) expondría datos personales de menores sin que la biblioteca tenga forma de detectarlo o mitigarlo.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Medio — imposibilidad de auditar acciones individuales, dificulta rendición de cuentas ante RNBP</t>
+          <t>Alto — exposición de datos personales de menores, con implicaciones bajo la Ley 1581 de 2012 de protección de datos personales</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Baja hoy (1 sola empleada), creciente si se contrata personal</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Medio</t>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Ninguno — el propio diseño del sistema (usuario único por biblioteca, no por persona) impide la atribución individual por diseño, según confirma el manual oficial.</t>
+          <t>No verificable desde la biblioteca: infraestructura tratada como 'caja negra' (Taller 4); Biteca no entregó información de cifrado ni de backups por restricciones contractuales; no se evidenció acuerdo de transmisión de datos entre la Alcaldía e IDECUT/Biteca (Taller 6, ítem 8).</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mientras el sistema no ofrezca usuarios individuales, documentar internamente (bitácora externa) quién realizó cada sesión de trabajo relevante.</t>
+          <t>Solicitar formalmente a Biteca/IDECUT y a la RNBP documentación sobre cifrado y cumplimiento de la Ley 1581 de 2012 para datos de menores, formalizar el acuerdo de transmisión con Biteca y capturar solo los campos estrictamente necesarios.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Bibliotecaria / RNBP</t>
+          <t>Alcaldía de Cogua / IDECUT-Biteca / RNBP</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -715,37 +715,37 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T6</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Base de Datos Koha y Base de Datos Llave del Saber</t>
+          <t>Catálogo público (OPAC) y app Nextbit; categorías y permisos de usuario en Koha</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Information Disclosure</t>
+          <t>Elevation of Privilege</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Ambas bases almacenan datos personales sensibles, incluyendo de menores de edad (categorías 'Niños 6-12' y 'Primera Infancia 0-5'), sin que el equipo tenga visibilidad de los controles de acceso y cifrado del proveedor externo.</t>
+          <t>El OPAC (cogua.bibliotecasidecut.com) y la app Nextbit ya exponen la instancia de Koha a internet. Una configuración incorrecta de permisos por categoría o de la separación entre la interfaz pública y la del personal podría permitir que un usuario común acceda a funciones administrativas.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Una filtración en la infraestructura del proveedor externo (RNBP o el hosting de Koha) expondría datos personales de menores sin que la biblioteca tenga forma de detectarlo o mitigarlo.</t>
+          <t>Un usuario afiliado, o alguien sin cuenta, descubre o adivina una ruta administrativa de Koha no protegida adecuadamente en el servidor y accede a funciones reservadas para el personal.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Alto — exposición de datos personales de menores, con implicaciones bajo la Ley 1581 de 2012 de protección de datos personales</t>
+          <t>Alto: un usuario no autorizado podría modificar el catálogo completo o los datos personales de otros afiliados, incluidos menores</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media: la superficie pública ya existe; no hay evidencia de los controles que Biteca aplica</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -755,17 +755,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>No verificable desde la biblioteca — infraestructura tratada como 'caja negra' (ya documentado en el Taller 4); sin evidencia pública de cifrado en reposo ni política de retención para datos de menores.</t>
+          <t>No verificable: Biteca no informó parches ni endurecimiento del OPAC (Taller 4: 'no informado'). El acceso del personal usa cuentas compartidas con permisos de edición.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Solicitar formalmente a RNBP y al proveedor de hosting de Koha documentación sobre cifrado y cumplimiento de la Ley 1581 de 2012 para datos de menores; capturar solo los campos estrictamente necesarios.</t>
+          <t>Solicitar a Biteca evidencia de separación de la interfaz pública y la del personal, de parches y de restricción de funciones administrativas; revisar internamente los permisos por rol (nunca solo en la interfaz).</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>RNBP / Proveedor de hosting Koha</t>
+          <t>Biteca / IDECUT (con seguimiento de la bibliotecaria)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -777,32 +777,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T7</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Conexión a Internet Local de la biblioteca</t>
+          <t>D3: Respuestas del formulario de inscripción (Microsoft Forms, cuenta creada por un estudiante)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Denial of Service</t>
+          <t>Information Disclosure</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Al ser el único canal hacia Koha y Llave del Saber a la vez, su caída impide tanto el registro de nuevos usuarios como la consulta de datos existentes durante toda la interrupción.</t>
+          <t>El formulario que recoge datos personales, de menores y datos sensibles (discapacidad) está alojado en una cuenta personal de un estudiante, fuera del control de la Alcaldía, que es la Responsable del tratamiento.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Falla del proveedor de internet local (o un incidente de disponibilidad en la infraestructura de Koha/Llave del Saber, fuera del control de la biblioteca) deja a la bibliotecaria sin poder atender afiliaciones ni préstamos.</t>
+          <t>La cuenta se compromete (phishing, contraseña débil, sin MFA documentado), el estudiante termina el servicio social y conserva o pierde el acceso, o comparte las respuestas por correo; la base de inscripciones se expone o se pierde.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Medio — interrupción del servicio al usuario final, sin pérdida de datos</t>
+          <t>Alto: exposición o pérdida de datos personales, sensibles y de menores, con consecuencia disciplinaria para los servidores responsables (Procuraduría)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -810,24 +810,24 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Medio</t>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Ninguno — conexión única sin respaldo (ya documentado en el mapa de infraestructura del Taller 4). El propio manual de Llave del Saber contempla este escenario: permite registrar actividades con fecha retroactiva 'cuando el servicio de internet no está disponible'.</t>
+          <t>Parcial: el nuevo aviso de privacidad cubre el consentimiento (Taller 6, ítems 1 y 2), pero no la custodia de la cuenta ni de las respuestas (ítems 8 y 11).</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Evaluar un enlace de respaldo de bajo costo (router 4G/5G) para continuidad mínima del servicio, tal como se recomendó en el Taller 4.</t>
+          <t>Trasladar el formulario y sus respuestas a una cuenta institucional de la Alcaldía con MFA; definir responsables y revocar accesos al terminar cada servicio social.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Bibliotecaria / Municipio</t>
+          <t>Bibliotecaria / Alcaldía de Cogua</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -839,60 +839,246 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T8</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Categorías y permisos de usuario en Koha (roles Administrativo, Docente, etc.)</t>
+          <t>Reportes y exportaciones de Koha (P1) desde cuentas compartidas</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>Information Disclosure</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Con cuentas compartidas, cualquier estudiante puede generar reportes y exportar la base de usuarios sin que quede registro de quién lo hizo.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Un estudiante exporta el listado de usuarios (con datos de menores) y lo guarda o envía fuera de la biblioteca; no hay forma de saber quién ni cuándo.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Alto: fuga de la base de usuarios sin trazabilidad (Taller 6, ítem 11, brecha de prioridad Alta)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Ninguno evidenciado: no existe restricción de reportes por rol ni registro individual de exportaciones.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Restringir los reportes y las exportaciones de Koha a la bibliotecaria y habilitar cuentas individuales para que cada exportación quede asociada a una persona.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Bibliotecaria</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Cuentas de Koha con permisos de edición compartidas con estudiantes (P1)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>Elevation of Privilege</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Si a futuro se habilita un portal público (OPAC) para usuarios/afiliados, como se propuso en el diagnóstico AS-IS previo, una configuración incorrecta de permisos por categoría podría permitir que un usuario común acceda a funciones administrativas.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Un usuario afiliado descubre o adivina una ruta administrativa de Koha no protegida adecuadamente en el backend y accede a funciones reservadas para el rol 'Administrativo'.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Alto — un usuario no autorizado podría modificar el catálogo completo o datos de otros afiliados</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Baja (no existe portal público todavía; riesgo latente para la fase TO-BE)</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Los estudiantes operan con los mismos permisos de edición de la bibliotecaria, que son más amplios de lo que su función de catalogación requiere (principio de mínimo privilegio).</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Un estudiante, por error o a propósito, edita o elimina registros de usuarios o cambia datos que solo debería modificar la bibliotecaria; una cuenta no dada de baja al terminar el servicio sigue activa.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Alto: alteración o pérdida de datos personales y del catálogo (Taller 6, ítem 9, brecha de prioridad Alta)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Ninguno: las dos cuentas con permisos de edición se comparten y no hay perfil restringido para estudiantes.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Crear cuentas individuales con perfil de catalogador restringido para los estudiantes, deshabilitarlas al terminar el servicio social y reservar la edición de usuarios a la bibliotecaria.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Bibliotecaria</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Doble registro manual de datos personales (Koha y Llave del Saber), transcritos desde las respuestas del formulario</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Tampering</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Al ingresarse manualmente el mismo dato dos veces sin validación cruzada automática, un error de digitación o una alteración intencional en una de las dos plataformas no es detectada por la otra.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Alguien con acceso a una de las dos plataformas, o a las respuestas del formulario, modifica un dato personal (ej. dirección o fecha de nacimiento) sin que exista mecanismo de reconciliación frente a las demás fuentes.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Medio — inconsistencia de datos personales entre sistemas; dificulta auditoría y reportes al Ministerio</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>No aplica de forma directa todavía — riesgo latente para cuando se implemente el canal digital de usuarios propuesto en el diagnóstico AS-IS.</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Si se implementa un portal público, revalidar los permisos por rol en el servidor (nunca solo en la interfaz) antes de habilitar cualquier acceso remoto.</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Equipo de desarrollo (fase TO-BE)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Ninguno automatizado: la reconciliación depende de una sola persona (cuello de botella ya diagnosticado en el Taller 4 de infraestructura). Supuesto por confirmar: la bibliotecaria transcribe las respuestas del formulario a ambas plataformas.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Definir un identificador único compartido (número de documento) y un proceso periódico de cruce de reportes entre ambas plataformas para detectar discrepancias.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Bibliotecaria</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Conexión a Internet Local de la biblioteca</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Denial of Service</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Al ser el único canal hacia Koha y Llave del Saber a la vez, su caída impide tanto el registro de nuevos usuarios como la consulta de datos existentes durante toda la interrupción.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Falla del proveedor de internet local (o un incidente de disponibilidad en la infraestructura de Koha/Llave del Saber, fuera del control de la biblioteca) deja a la bibliotecaria sin poder atender afiliaciones ni préstamos.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Medio — interrupción del servicio al usuario final, sin pérdida de datos</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Ninguno: conexión única sin respaldo (Taller 4, observaciones adicionales; se lleva a la zona 'Biblioteca de Cogua' del mapa y a la tabla de diagnóstico). El propio manual de Llave del Saber contempla este escenario: permite registrar actividades con fecha retroactiva 'cuando el servicio de internet no está disponible'.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Evaluar un enlace de respaldo de bajo costo (router 4G/5G) para continuidad mínima del servicio, tal como se recomendó en el Taller 4.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Bibliotecaria / Municipio</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>

</xml_diff>